<commit_message>
docs(gate): R4-W2 통합 근거와 WBS 반영
변경: R4-W2를 MERGED_DEV로 전환하고 평가 원장·Markdown/공식 XLSX WBS·R1 일일보고에 제어 흐름과 검증 근거를 연결했다.
검증: pipeline 8건·integration 16건, dev CI run 30606915908, 문서 정책·WBS·보고서·XLSX 렌더링과 구조 검증 PASS.
</commit_message>
<xml_diff>
--- a/docs/deliverables/02_WBS_29기_3팀.xlsx
+++ b/docs/deliverables/02_WBS_29기_3팀.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="갠트 차트 템플릿" sheetId="1" r:id="R88c0c307107b4720"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="갠트 차트 템플릿" sheetId="1" r:id="R8448e77e2a3c40a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6971,7 +6971,7 @@
         <x:v>4.5</x:v>
       </x:c>
       <x:c r="C63" s="267" t="str">
-        <x:v>[진행] R4-04 Router·Template Binding
+        <x:v>[완료] R4-04 Router·Template Binding
 산출물: route decision · 우선순위: 높음</x:v>
       </x:c>
       <x:c r="D63" s="267" t="str">
@@ -6988,7 +6988,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="H63" s="270" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I63" s="271"/>
       <x:c r="J63" s="271"/>
@@ -7056,7 +7056,7 @@
         <x:v>4.6</x:v>
       </x:c>
       <x:c r="C64" s="267" t="str">
-        <x:v>[진행] R4-05 Controller 고정 상태 머신
+        <x:v>[완료] R4-05 Controller 고정 상태 머신
 산출물: transition table · 우선순위: 높음</x:v>
       </x:c>
       <x:c r="D64" s="267" t="str">
@@ -7073,7 +7073,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="H64" s="270" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I64" s="271"/>
       <x:c r="J64" s="271"/>
@@ -7141,7 +7141,7 @@
         <x:v>4.7</x:v>
       </x:c>
       <x:c r="C65" s="267" t="str">
-        <x:v>[대기] R4-06 Context Registry·Builder
+        <x:v>[완료] R4-06 Context Registry·Builder
 산출물: versioned Context Package · 우선순위: 높음</x:v>
       </x:c>
       <x:c r="D65" s="267" t="str">
@@ -7158,7 +7158,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="H65" s="270" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I65" s="271"/>
       <x:c r="J65" s="271"/>
@@ -7226,7 +7226,7 @@
         <x:v>4.8</x:v>
       </x:c>
       <x:c r="C66" s="267" t="str">
-        <x:v>[대기] R4-07 G1 Context Gate
+        <x:v>[완료] R4-07 G1 Context Gate
 산출물: decision·evidence · 우선순위: 높음</x:v>
       </x:c>
       <x:c r="D66" s="267" t="str">
@@ -7243,7 +7243,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="H66" s="270" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I66" s="271"/>
       <x:c r="J66" s="271"/>
@@ -7311,7 +7311,7 @@
         <x:v>4.9</x:v>
       </x:c>
       <x:c r="C67" s="267" t="str">
-        <x:v>[대기] R4-08 R3 Node typed client
+        <x:v>[완료] R4-08 R3 Node typed client
 산출물: model client·오류 처리 · 우선순위: 높음</x:v>
       </x:c>
       <x:c r="D67" s="267" t="str">
@@ -7328,7 +7328,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="H67" s="270" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I67" s="271"/>
       <x:c r="J67" s="271"/>
@@ -7396,7 +7396,7 @@
         <x:v>4.10</x:v>
       </x:c>
       <x:c r="C68" s="267" t="str">
-        <x:v>[대기] R4-09 G2 SQL Policy Gate
+        <x:v>[완료] R4-09 G2 SQL Policy Gate
 산출물: AST·policy decision · 우선순위: 높음</x:v>
       </x:c>
       <x:c r="D68" s="267" t="str">
@@ -7413,7 +7413,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="H68" s="270" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I68" s="271"/>
       <x:c r="J68" s="271"/>
@@ -7481,7 +7481,7 @@
         <x:v>4.11</x:v>
       </x:c>
       <x:c r="C69" s="267" t="str">
-        <x:v>[대기] R4-10 Node 2′·G2′ 수정 1회 통제
+        <x:v>[완료] R4-10 Node 2′·G2′ 수정 1회 통제
 산출물: repair counter · 우선순위: 높음</x:v>
       </x:c>
       <x:c r="D69" s="267" t="str">
@@ -7498,7 +7498,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="H69" s="270" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I69" s="271"/>
       <x:c r="J69" s="271"/>
@@ -7566,7 +7566,7 @@
         <x:v>4.12</x:v>
       </x:c>
       <x:c r="C70" s="267" t="str">
-        <x:v>[대기] R4-11 R2 Trino 실행 lifecycle 통제
+        <x:v>[완료] R4-11 R2 Trino 실행 lifecycle 통제
 산출물: pass token·timeout·cancel · 우선순위: 높음</x:v>
       </x:c>
       <x:c r="D70" s="267" t="str">
@@ -7583,7 +7583,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="H70" s="270" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I70" s="271"/>
       <x:c r="J70" s="271"/>
@@ -7651,7 +7651,7 @@
         <x:v>4.13</x:v>
       </x:c>
       <x:c r="C71" s="267" t="str">
-        <x:v>[대기] R4-12 Result Shaper·G3
+        <x:v>[완료] R4-12 Result Shaper·G3
 산출물: shaped result·evidence · 우선순위: 높음</x:v>
       </x:c>
       <x:c r="D71" s="267" t="str">
@@ -7668,7 +7668,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="H71" s="270" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I71" s="271"/>
       <x:c r="J71" s="271"/>
@@ -7736,7 +7736,7 @@
         <x:v>4.14</x:v>
       </x:c>
       <x:c r="C72" s="267" t="str">
-        <x:v>[대기] R4-13 Node 3·승인 후 수정 불가 Artifact
+        <x:v>[완료] R4-13 Node 3·승인 후 수정 불가 Artifact
 산출물: artifact contract · 우선순위: 높음</x:v>
       </x:c>
       <x:c r="D72" s="267" t="str">
@@ -7753,7 +7753,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="H72" s="270" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I72" s="271"/>
       <x:c r="J72" s="271"/>
@@ -7906,7 +7906,7 @@
         <x:v>4.16</x:v>
       </x:c>
       <x:c r="C74" s="267" t="str">
-        <x:v>[대기] R4-15 Audit·Trace·관측
+        <x:v>[완료] R4-15 Audit·Trace·관측
 산출물: linked request trace · 우선순위: 높음</x:v>
       </x:c>
       <x:c r="D74" s="267" t="str">
@@ -7923,7 +7923,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="H74" s="270" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I74" s="271"/>
       <x:c r="J74" s="271"/>

</xml_diff>